<commit_message>
Simplify H2 and internal link cell format in batch 1-6 workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011yk4rjpNDYyzEGMQKf1aSb
</commit_message>
<xml_diff>
--- a/output/motherandbeyond_H2_Research_Batch1-6.xlsx
+++ b/output/motherandbeyond_H2_Research_Batch1-6.xlsx
@@ -513,11 +513,11 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Bintik Merah DBD dan Biang Keringat? (AI Citation Score: 9/10 | Type: Definitional)
-2. 5 Perbedaan Bintik Merah DBD dan Biang Keringat yang Mudah Dikenali (AI Citation Score: 10/10 | Type: Comparative)
-3. Cara Cek Bintik Merah DBD di Rumah: Uji Tekan dan Uji Regang Kulit (AI Citation Score: 9/10 | Type: Procedural)
-4. Kapan Bintik Merah DBD Muncul dan Gejala Penyerta yang Perlu Diwaspadai (AI Citation Score: 9/10 | Type: Factual)
-5. Langkah Penanganan Awal dan Tanda Anak Harus Segera Dibawa ke Dokter (AI Citation Score: 8/10 | Type: Procedural)</t>
+          <t>1. Apa Itu Bintik Merah DBD dan Biang Keringat?
+2. 5 Perbedaan Bintik Merah DBD dan Biang Keringat yang Mudah Dikenali
+3. Cara Cek Bintik Merah DBD di Rumah: Uji Tekan dan Uji Regang Kulit
+4. Kapan Bintik Merah DBD Muncul dan Gejala Penyerta yang Perlu Diwaspadai
+5. Langkah Penanganan Awal dan Tanda Anak Harus Segera Dibawa ke Dokter</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -534,12 +534,12 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: gejala DBD pada anak yang perlu diwaspadai → URL: https://motherandbeyond.id/read/20743/waspada-demam-berdarah-dengue-kenali-gejala-dbd-pada-anak
-2. Anchor: perbedaan campak dan alergi → URL: https://motherandbeyond.id/read/25745/ini-perbedaan-campak-dan-alergi-yang-perlu-moms-pahami
-3. Anchor: bentol berair pada kulit bayi → URL: https://motherandbeyond.id/read/26951/bentol-berair-pada-kulit-bayi-ini-penyebab-dan-cara-mengatasinya
-4. Anchor: anak demam tapi tangan dan kaki dingin → URL: https://motherandbeyond.id/read/26753/5-cara-mengatasi-anak-demam-tapi-tangan-dan-kaki-dingin
-5. Anchor: kejang demam pada bayi → URL: https://motherandbeyond.id/read/22211/kejang-demam-pada-bayi-ini-yang-perlu-anda-perhatikan
-6. Anchor: makanan dan minuman yang bantu turunkan demam anak → URL: https://motherandbeyond.id/read/17871/7-makanan-dan-minuman-yang-bantu-turunkan-demam-anak</t>
+          <t>1. https://motherandbeyond.id/read/20743/waspada-demam-berdarah-dengue-kenali-gejala-dbd-pada-anak
+2. https://motherandbeyond.id/read/25745/ini-perbedaan-campak-dan-alergi-yang-perlu-moms-pahami
+3. https://motherandbeyond.id/read/26951/bentol-berair-pada-kulit-bayi-ini-penyebab-dan-cara-mengatasinya
+4. https://motherandbeyond.id/read/26753/5-cara-mengatasi-anak-demam-tapi-tangan-dan-kaki-dingin
+5. https://motherandbeyond.id/read/22211/kejang-demam-pada-bayi-ini-yang-perlu-anda-perhatikan
+6. https://motherandbeyond.id/read/17871/7-makanan-dan-minuman-yang-bantu-turunkan-demam-anak</t>
         </is>
       </c>
     </row>
@@ -559,11 +559,11 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>1. Makna Sholawat sebagai Pengantar Tidur Bayi dalam Tradisi Islam (AI Citation Score: 8/10 | Type: Definitional)
-2. Kumpulan Sholawat Pengantar Tidur Bayi: Arab, Latin, dan Artinya (AI Citation Score: 10/10 | Type: Recommendation)
-3. Sholawat Nariyah, Badar, dan Jibril: Mana yang Cocok untuk Bayi Rewel? (AI Citation Score: 8/10 | Type: Comparative)
-4. Cara Melantunkan Sholawat agar Bayi Cepat Tenang dan Tidur Nyenyak (AI Citation Score: 8/10 | Type: Procedural)
-5. Manfaat Rutin Bersholawat Menjelang Tidur bagi Bayi dan Ibu (AI Citation Score: 7/10 | Type: Factual)</t>
+          <t>1. Makna Sholawat sebagai Pengantar Tidur Bayi dalam Tradisi Islam
+2. Kumpulan Sholawat Pengantar Tidur Bayi: Arab, Latin, dan Artinya
+3. Sholawat Nariyah, Badar, dan Jibril: Mana yang Cocok untuk Bayi Rewel?
+4. Cara Melantunkan Sholawat agar Bayi Cepat Tenang dan Tidur Nyenyak
+5. Manfaat Rutin Bersholawat Menjelang Tidur bagi Bayi dan Ibu</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
@@ -580,11 +580,11 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: doa agar bayi tidur nyenyak dan tidak rewel → URL: https://motherandbeyond.id/read/27900/bacaan-doa-agar-bayi-tidur-nyenyak-dan-tidak-rewel
-2. Anchor: sleep regression pada bayi → URL: https://motherandbeyond.id/read/23510/mengenal-sleep-regression-gangguan-tidur-pada-bayi
-3. Anchor: dongeng sebelum tidur yang singkat → URL: https://motherandbeyond.id/read/25388/dongeng-sebelum-tidur-yang-singkat-dan-penuh-makna-untuk-anak
-4. Anchor: cara mengatasi bayi yang tidur miring → URL: https://motherandbeyond.id/read/26780/moms-ini-cara-mengatasi-bayi-yang-tidur-miring
-5. Anchor: bayi tidur terus, normal atau tidak → URL: https://motherandbeyond.id/read/16721/bayi-tidur-terus-ini-penyebab-dan-cara-mengatasinya</t>
+          <t>1. https://motherandbeyond.id/read/27900/bacaan-doa-agar-bayi-tidur-nyenyak-dan-tidak-rewel
+2. https://motherandbeyond.id/read/23510/mengenal-sleep-regression-gangguan-tidur-pada-bayi
+3. https://motherandbeyond.id/read/25388/dongeng-sebelum-tidur-yang-singkat-dan-penuh-makna-untuk-anak
+4. https://motherandbeyond.id/read/26780/moms-ini-cara-mengatasi-bayi-yang-tidur-miring
+5. https://motherandbeyond.id/read/16721/bayi-tidur-terus-ini-penyebab-dan-cara-mengatasinya</t>
         </is>
       </c>
     </row>
@@ -604,11 +604,11 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>1. Makna Hari Ibu 22 Desember di Indonesia dan Mengapa Ucapan Itu Penting (AI Citation Score: 8/10 | Type: Factual)
-2. Ucapan Hari Ibu Singkat yang Menyentuh Hati untuk Caption dan Pesan WhatsApp (AI Citation Score: 10/10 | Type: Recommendation)
-3. Ucapan Hari Ibu Islami Penuh Doa untuk Ibu Tercinta (AI Citation Score: 9/10 | Type: Recommendation)
-4. Ucapan Hari Ibu untuk Ibu yang Sudah Meninggal (AI Citation Score: 9/10 | Type: Recommendation)
-5. Cara Menulis Ucapan Hari Ibu yang Personal dan Tidak Klise (AI Citation Score: 7/10 | Type: Procedural)</t>
+          <t>1. Makna Hari Ibu 22 Desember di Indonesia dan Mengapa Ucapan Itu Penting
+2. Ucapan Hari Ibu Singkat yang Menyentuh Hati untuk Caption dan Pesan WhatsApp
+3. Ucapan Hari Ibu Islami Penuh Doa untuk Ibu Tercinta
+4. Ucapan Hari Ibu untuk Ibu yang Sudah Meninggal
+5. Cara Menulis Ucapan Hari Ibu yang Personal dan Tidak Klise</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -625,10 +625,10 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: kata-kata ibu rindu anak → URL: https://motherandbeyond.id/read/27467/50-kata-kata-ibu-rindu-anak-yang-menyentuh-dan-penuh-makna
-2. Anchor: ucapan ulang tahun untuk mertua → URL: https://motherandbeyond.id/read/26888/30-ucapan-ulang-tahun-untuk-mertua-yang-penuh-makna
-3. Anchor: arti mimpi ibu meninggal → URL: https://motherandbeyond.id/read/28197/jangan-panik-ini-arti-mimpi-ibu-meninggal-yang-perlu-moms-tahu
-4. Anchor: ucapan ulang tahun untuk istri tercinta → URL: https://motherandbeyond.id/read/24620/18-ucapan-ulang-tahun-yang-romantis-untuk-istri-tercinta-dijamin-makin-disayang</t>
+          <t>1. https://motherandbeyond.id/read/27467/50-kata-kata-ibu-rindu-anak-yang-menyentuh-dan-penuh-makna
+2. https://motherandbeyond.id/read/26888/30-ucapan-ulang-tahun-untuk-mertua-yang-penuh-makna
+3. https://motherandbeyond.id/read/28197/jangan-panik-ini-arti-mimpi-ibu-meninggal-yang-perlu-moms-tahu
+4. https://motherandbeyond.id/read/24620/18-ucapan-ulang-tahun-yang-romantis-untuk-istri-tercinta-dijamin-makin-disayang</t>
         </is>
       </c>
     </row>
@@ -648,11 +648,11 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu SIDS pada Bayi dan Usia Berapa Risikonya Paling Tinggi? (AI Citation Score: 10/10 | Type: Definitional)
-2. Penyebab dan Faktor Risiko SIDS yang Perlu Orang Tua Ketahui (AI Citation Score: 9/10 | Type: Factual)
-3. Benarkah Tidur Tengkurap Memicu SIDS? Ini Posisi Tidur Bayi yang Aman (AI Citation Score: 9/10 | Type: Comparative)
-4. Cara Mencegah SIDS: Checklist Tidur Aman untuk Bayi (AI Citation Score: 10/10 | Type: Procedural)
-5. Perbedaan SIDS dan SUID serta Kapan Harus Konsultasi ke Dokter (AI Citation Score: 7/10 | Type: Comparative)</t>
+          <t>1. Apa Itu SIDS pada Bayi dan Usia Berapa Risikonya Paling Tinggi?
+2. Penyebab dan Faktor Risiko SIDS yang Perlu Orang Tua Ketahui
+3. Benarkah Tidur Tengkurap Memicu SIDS? Ini Posisi Tidur Bayi yang Aman
+4. Cara Mencegah SIDS: Checklist Tidur Aman untuk Bayi
+5. Perbedaan SIDS dan SUID serta Kapan Harus Konsultasi ke Dokter</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -669,11 +669,11 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: cara mengatasi bayi yang tidur miring → URL: https://motherandbeyond.id/read/26780/moms-ini-cara-mengatasi-bayi-yang-tidur-miring
-2. Anchor: cara aman melatih bayi tengkurap → URL: https://motherandbeyond.id/read/26469/cara-aman-melatih-bayi-tengkurap-dan-manfaatnya
-3. Anchor: sleep regression pada bayi → URL: https://motherandbeyond.id/read/23510/mengenal-sleep-regression-gangguan-tidur-pada-bayi
-4. Anchor: bayi tidur terus, apakah normal → URL: https://motherandbeyond.id/read/16721/bayi-tidur-terus-ini-penyebab-dan-cara-mengatasinya
-5. Anchor: cara aman membangunkan bayi → URL: https://motherandbeyond.id/read/26850/8-cara-aman-membangunkan-bayi-yang-tidur-terus</t>
+          <t>1. https://motherandbeyond.id/read/26780/moms-ini-cara-mengatasi-bayi-yang-tidur-miring
+2. https://motherandbeyond.id/read/26469/cara-aman-melatih-bayi-tengkurap-dan-manfaatnya
+3. https://motherandbeyond.id/read/23510/mengenal-sleep-regression-gangguan-tidur-pada-bayi
+4. https://motherandbeyond.id/read/16721/bayi-tidur-terus-ini-penyebab-dan-cara-mengatasinya
+5. https://motherandbeyond.id/read/26850/8-cara-aman-membangunkan-bayi-yang-tidur-terus</t>
         </is>
       </c>
     </row>
@@ -693,11 +693,11 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Bedak Salicyl dan Kandungannya? (AI Citation Score: 8/10 | Type: Definitional)
-2. Apakah Bedak Salicyl Aman untuk Bayi? Ini Batas Usia yang Dianjurkan (AI Citation Score: 10/10 | Type: Factual)
-3. Manfaat Bedak Salicyl untuk Biang Keringat dan Gatal pada Kulit Anak (AI Citation Score: 8/10 | Type: Factual)
-4. Cara Pakai Bedak Salicyl yang Aman dan Efek Samping yang Perlu Diwaspadai (AI Citation Score: 9/10 | Type: Procedural)
-5. Alternatif Perawatan Biang Keringat untuk Bayi di Bawah 2 Tahun (AI Citation Score: 8/10 | Type: Recommendation)</t>
+          <t>1. Apa Itu Bedak Salicyl dan Kandungannya?
+2. Apakah Bedak Salicyl Aman untuk Bayi? Ini Batas Usia yang Dianjurkan
+3. Manfaat Bedak Salicyl untuk Biang Keringat dan Gatal pada Kulit Anak
+4. Cara Pakai Bedak Salicyl yang Aman dan Efek Samping yang Perlu Diwaspadai
+5. Alternatif Perawatan Biang Keringat untuk Bayi di Bawah 2 Tahun</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -714,10 +714,9 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: bentol berair pada kulit bayi → URL: https://motherandbeyond.id/read/26951/bentol-berair-pada-kulit-bayi-ini-penyebab-dan-cara-mengatasinya
-2. Anchor: perbedaan campak dan alergi → URL: https://motherandbeyond.id/read/25745/ini-perbedaan-campak-dan-alergi-yang-perlu-moms-pahami
-3. Anchor: gejala DBD pada anak → URL: https://motherandbeyond.id/read/20743/waspada-demam-berdarah-dengue-kenali-gejala-dbd-pada-anak
-Limited relevant internal link available from Ahrefs export.</t>
+          <t>1. https://motherandbeyond.id/read/26951/bentol-berair-pada-kulit-bayi-ini-penyebab-dan-cara-mengatasinya
+2. https://motherandbeyond.id/read/25745/ini-perbedaan-campak-dan-alergi-yang-perlu-moms-pahami
+3. https://motherandbeyond.id/read/20743/waspada-demam-berdarah-dengue-kenali-gejala-dbd-pada-anak</t>
         </is>
       </c>
     </row>
@@ -737,11 +736,11 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Akta Kelahiran dan Kapan Batas Waktu Pengurusannya? (AI Citation Score: 8/10 | Type: Definitional)
-2. Syarat Dokumen Membuat Akta Kelahiran Anak (AI Citation Score: 10/10 | Type: Factual)
-3. Cara Membuat Akta Kelahiran Secara Offline di Disdukcapil (AI Citation Score: 9/10 | Type: Procedural)
-4. Cara Membuat Akta Kelahiran Online Lewat Aplikasi Dukcapil (AI Citation Score: 10/10 | Type: Procedural)
-5. Mengurus Akta Kelahiran Terlambat dan Kondisi Khusus (SPTJM, Tanpa Buku Nikah) (AI Citation Score: 8/10 | Type: Comparative)</t>
+          <t>1. Apa Itu Akta Kelahiran dan Kapan Batas Waktu Pengurusannya?
+2. Syarat Dokumen Membuat Akta Kelahiran Anak
+3. Cara Membuat Akta Kelahiran Secara Offline di Disdukcapil
+4. Cara Membuat Akta Kelahiran Online Lewat Aplikasi Dukcapil
+5. Mengurus Akta Kelahiran Terlambat dan Kondisi Khusus (SPTJM, Tanpa Buku Nikah)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -758,10 +757,9 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: ucapan kelahiran bayi laki-laki penuh doa → URL: https://motherandbeyond.id/read/27602/50-ucapan-kelahiran-bayi-laki-laki-penuh-doa-dan-makna
-2. Anchor: nama bayi laki-laki islam modern → URL: https://motherandbeyond.id/read/27384/150-nama-bayi-laki-laki-islam-modern-beserta-artinya
-3. Anchor: pantangan ibu baru melahirkan sebelum 40 hari → URL: https://motherandbeyond.id/read/26873/pantangan-ibu-baru-melahirkan-sebelum-40-hari-mitos-atau-fakta-medis
-Limited relevant internal link available from Ahrefs export.</t>
+          <t>1. https://motherandbeyond.id/read/27602/50-ucapan-kelahiran-bayi-laki-laki-penuh-doa-dan-makna
+2. https://motherandbeyond.id/read/27384/150-nama-bayi-laki-laki-islam-modern-beserta-artinya
+3. https://motherandbeyond.id/read/26873/pantangan-ibu-baru-melahirkan-sebelum-40-hari-mitos-atau-fakta-medis</t>
         </is>
       </c>
     </row>
@@ -781,11 +779,11 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1. Apa yang Terjadi pada Tubuh Ibu dan Janin di Usia Kehamilan 5 Bulan? (AI Citation Score: 8/10 | Type: Definitional)
-2. 7 Ciri-Ciri Hamil 5 Bulan yang Sehat yang Perlu Bunda Kenali (AI Citation Score: 10/10 | Type: Factual)
-3. Perkembangan Janin Usia 5 Bulan: Ukuran, Berat, dan Gerakan (AI Citation Score: 9/10 | Type: Factual)
-4. Hamil 5 Bulan Normal vs Tanda Bahaya yang Harus Segera Diperiksakan (AI Citation Score: 9/10 | Type: Comparative)
-5. Tips Menjaga Kehamilan 5 Bulan Tetap Sehat: Nutrisi, Aktivitas, dan Kontrol Rutin (AI Citation Score: 8/10 | Type: Procedural)</t>
+          <t>1. Apa yang Terjadi pada Tubuh Ibu dan Janin di Usia Kehamilan 5 Bulan?
+2. 7 Ciri-Ciri Hamil 5 Bulan yang Sehat yang Perlu Bunda Kenali
+3. Perkembangan Janin Usia 5 Bulan: Ukuran, Berat, dan Gerakan
+4. Hamil 5 Bulan Normal vs Tanda Bahaya yang Harus Segera Diperiksakan
+5. Tips Menjaga Kehamilan 5 Bulan Tetap Sehat: Nutrisi, Aktivitas, dan Kontrol Rutin</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -802,12 +800,12 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: bentuk janin 5 bulan di USG → URL: https://motherandbeyond.id/read/28066/seperti-apa-bentuk-janin-5-bulan-di-usg-ini-penjelasannya-moms
-2. Anchor: hamil 5 bulan tapi belum merasakan gerakan janin → URL: https://motherandbeyond.id/read/25789/hamil-5-bulan-tapi-belum-merasakan-gerakan-janin-normalkah
-3. Anchor: perkembangan janin di kehamilan 5 bulan → URL: https://motherandbeyond.id/read/10681/perkembangan-janin-di-kehamilan-5-bulan
-4. Anchor: ciri janin sehat dalam kandungan → URL: https://motherandbeyond.id/read/23860/bumil-wajib-tahu-ini-6-ciri-janin-sehat-dalam-kandungan
-5. Anchor: keputihan saat hamil trimester 2 → URL: https://motherandbeyond.id/read/26891/ini-penyebab-dan-cara-mengatasi-keputihan-saat-hamil-trimester-2
-6. Anchor: nyeri perut saat hamil trimester 2 → URL: https://motherandbeyond.id/read/25751/nyeri-perut-normal-terjadi-saat-hamil-di-trimester-2-ini-penyebabnya</t>
+          <t>1. https://motherandbeyond.id/read/28066/seperti-apa-bentuk-janin-5-bulan-di-usg-ini-penjelasannya-moms
+2. https://motherandbeyond.id/read/25789/hamil-5-bulan-tapi-belum-merasakan-gerakan-janin-normalkah
+3. https://motherandbeyond.id/read/10681/perkembangan-janin-di-kehamilan-5-bulan
+4. https://motherandbeyond.id/read/23860/bumil-wajib-tahu-ini-6-ciri-janin-sehat-dalam-kandungan
+5. https://motherandbeyond.id/read/26891/ini-penyebab-dan-cara-mengatasi-keputihan-saat-hamil-trimester-2
+6. https://motherandbeyond.id/read/25751/nyeri-perut-normal-terjadi-saat-hamil-di-trimester-2-ini-penyebabnya</t>
         </is>
       </c>
     </row>
@@ -827,11 +825,11 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>1. Manfaat Tebak-Tebakan Hewan untuk Perkembangan Anak SD (AI Citation Score: 7/10 | Type: Factual)
-2. Tebak-Tebakan Hewan Berdasarkan Ciri Fisik dan Suaranya (AI Citation Score: 9/10 | Type: Recommendation)
-3. Tebak-Tebakan Hewan Lucu dan Plesetan yang Bikin Anak Tertawa (AI Citation Score: 9/10 | Type: Recommendation)
-4. Tebak-Tebakan Hewan Edukatif: Habitat, Makanan, dan Fakta Unik (AI Citation Score: 8/10 | Type: Recommendation)
-5. Cara Seru Memainkan Tebak-Tebakan Hewan di Rumah dan di Kelas (AI Citation Score: 7/10 | Type: Procedural)</t>
+          <t>1. Manfaat Tebak-Tebakan Hewan untuk Perkembangan Anak SD
+2. Tebak-Tebakan Hewan Berdasarkan Ciri Fisik dan Suaranya
+3. Tebak-Tebakan Hewan Lucu dan Plesetan yang Bikin Anak Tertawa
+4. Tebak-Tebakan Hewan Edukatif: Habitat, Makanan, dan Fakta Unik
+5. Cara Seru Memainkan Tebak-Tebakan Hewan di Rumah dan di Kelas</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -848,10 +846,10 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: 100 soal pengetahuan umum SD dan jawabannya → URL: https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
-2. Anchor: kata-kata motivasi untuk anak SD → URL: https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
-3. Anchor: dongeng sebelum tidur yang singkat → URL: https://motherandbeyond.id/read/25388/dongeng-sebelum-tidur-yang-singkat-dan-penuh-makna-untuk-anak
-4. Anchor: ide menu bekal sekolah anak SD → URL: https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi</t>
+          <t>1. https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
+2. https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
+3. https://motherandbeyond.id/read/25388/dongeng-sebelum-tidur-yang-singkat-dan-penuh-makna-untuk-anak
+4. https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi</t>
         </is>
       </c>
     </row>
@@ -871,11 +869,11 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>1. Tips Memilih Kado yang Tepat untuk Anak Laki-Laki 7 Tahun (AI Citation Score: 8/10 | Type: Procedural)
-2. Rekomendasi Kado Edukatif untuk Anak Laki-Laki 7 Tahun (AI Citation Score: 10/10 | Type: Recommendation)
-3. Ide Kado untuk Anak Aktif dan Suka Kegiatan Outdoor (AI Citation Score: 8/10 | Type: Recommendation)
-4. Kado Murah di Bawah Rp100 Ribu yang Tetap Berkesan (AI Citation Score: 9/10 | Type: Recommendation)
-5. Perbandingan Kado Berdasarkan Minat Anak: Tabel Harga dan Manfaat (AI Citation Score: 8/10 | Type: Comparative)</t>
+          <t>1. Tips Memilih Kado yang Tepat untuk Anak Laki-Laki 7 Tahun
+2. Rekomendasi Kado Edukatif untuk Anak Laki-Laki 7 Tahun
+3. Ide Kado untuk Anak Aktif dan Suka Kegiatan Outdoor
+4. Kado Murah di Bawah Rp100 Ribu yang Tetap Berkesan
+5. Perbandingan Kado Berdasarkan Minat Anak: Tabel Harga dan Manfaat</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -892,11 +890,11 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: kado untuk anak laki-laki 4 tahun → URL: https://motherandbeyond.id/read/26685/bingung-cari-kado-untuk-anak-laki-laki-4-tahun-ini-pilihan-terbaiknya
-2. Anchor: ucapan ulang tahun untuk anak laki-laki → URL: https://motherandbeyond.id/read/27213/50-ucapan-ulang-tahun-untuk-anak-laki-laki-yang-menyentuh-hati
-3. Anchor: kado bayi yang bermanfaat jangka panjang → URL: https://motherandbeyond.id/read/27898/10-kado-bayi-yang-bermanfaat-untuk-jangka-panjang-sampai-ia-besar
-4. Anchor: manfaat pop it fidget toy → URL: https://motherandbeyond.id/read/23087/bukan-mainan-biasa-ini-manfaat-dari-pop-it-fidget-toy-buat-anak
-5. Anchor: model rambut anak cowok terbaru → URL: https://motherandbeyond.id/read/28709/15-model-rambut-anak-cowok-terbaru-rapi-keren-dan-sesuai-aturan-sekolah</t>
+          <t>1. https://motherandbeyond.id/read/26685/bingung-cari-kado-untuk-anak-laki-laki-4-tahun-ini-pilihan-terbaiknya
+2. https://motherandbeyond.id/read/27213/50-ucapan-ulang-tahun-untuk-anak-laki-laki-yang-menyentuh-hati
+3. https://motherandbeyond.id/read/27898/10-kado-bayi-yang-bermanfaat-untuk-jangka-panjang-sampai-ia-besar
+4. https://motherandbeyond.id/read/23087/bukan-mainan-biasa-ini-manfaat-dari-pop-it-fidget-toy-buat-anak
+5. https://motherandbeyond.id/read/28709/15-model-rambut-anak-cowok-terbaru-rapi-keren-dan-sesuai-aturan-sekolah</t>
         </is>
       </c>
     </row>
@@ -916,11 +914,11 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>1. Berapa Ukuran Kaki Normal Anak Usia 3 Tahun? (AI Citation Score: 10/10 | Type: Factual)
-2. Tabel Konversi Ukuran Kaki ke Ukuran Sepatu Anak (EU, US, UK) (AI Citation Score: 10/10 | Type: Comparative)
-3. Cara Mengukur Kaki Anak dengan Benar di Rumah (AI Citation Score: 9/10 | Type: Procedural)
-4. Tips Memilih Sepatu yang Pas dan Sehat untuk Anak 3 Tahun (AI Citation Score: 8/10 | Type: Procedural)
-5. Seberapa Sering Ukuran Kaki Anak Perlu Dicek Ulang? (AI Citation Score: 8/10 | Type: Factual)</t>
+          <t>1. Berapa Ukuran Kaki Normal Anak Usia 3 Tahun?
+2. Tabel Konversi Ukuran Kaki ke Ukuran Sepatu Anak (EU, US, UK)
+3. Cara Mengukur Kaki Anak dengan Benar di Rumah
+4. Tips Memilih Sepatu yang Pas dan Sehat untuk Anak 3 Tahun
+5. Seberapa Sering Ukuran Kaki Anak Perlu Dicek Ulang?</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -937,10 +935,9 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: telapak tangan dan kaki anak panas → URL: https://motherandbeyond.id/read/27605/telapak-tangan-dan-kaki-anak-panas-ini-penyebab-dan-cara-mengatasinya
-2. Anchor: penyebab telapak kaki pecah-pecah → URL: https://motherandbeyond.id/read/24423/penyebab-telapak-kaki-pecah-pecah-dan-cara-mudah-mengatasinya
-3. Anchor: ciri anak hiperaktif usia 2 tahun → URL: https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun
-Limited relevant internal link available from Ahrefs export.</t>
+          <t>1. https://motherandbeyond.id/read/27605/telapak-tangan-dan-kaki-anak-panas-ini-penyebab-dan-cara-mengatasinya
+2. https://motherandbeyond.id/read/24423/penyebab-telapak-kaki-pecah-pecah-dan-cara-mudah-mengatasinya
+3. https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun</t>
         </is>
       </c>
     </row>
@@ -960,11 +957,11 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1. Kenapa Banyak Nenek Muda Kini Pilih Panggilan yang Lebih Gaul? (AI Citation Score: 7/10 | Type: Factual)
-2. Daftar Panggilan Nenek Gaul yang Unik dan Kekinian (AI Citation Score: 10/10 | Type: Recommendation)
-3. Panggilan Nenek dari Berbagai Bahasa dan Budaya (AI Citation Score: 8/10 | Type: Recommendation)
-4. Pasangan Panggilan Nenek dan Kakek yang Serasi (AI Citation Score: 8/10 | Type: Recommendation)
-5. Tips Memilih Panggilan Nenek yang Mudah Diucapkan Si Kecil (AI Citation Score: 7/10 | Type: Procedural)</t>
+          <t>1. Kenapa Banyak Nenek Muda Kini Pilih Panggilan yang Lebih Gaul?
+2. Daftar Panggilan Nenek Gaul yang Unik dan Kekinian
+3. Panggilan Nenek dari Berbagai Bahasa dan Budaya
+4. Pasangan Panggilan Nenek dan Kakek yang Serasi
+5. Tips Memilih Panggilan Nenek yang Mudah Diucapkan Si Kecil</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -981,10 +978,10 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: ide panggilan kakek yang unik dan kekinian → URL: https://motherandbeyond.id/read/28719/ide-panggilan-kakek-yang-unik-dan-kekinian-untuk-si-kecil
-2. Anchor: nama panggilan tante aesthetic dan kekinian → URL: https://motherandbeyond.id/read/28659/30-rekomendasi-nama-panggilan-tante-aesthetic-dan-kekinian
-3. Anchor: ide panggilan sayang yang unik untuk pasangan → URL: https://motherandbeyond.id/read/27740/ide-panggilan-sayang-yang-unik-dan-langka-untuk-pasangan
-4. Anchor: panggilan sayang unik selebriti → URL: https://motherandbeyond.id/read/23681/deretan-panggilan-sayang-unik-selebriti-untuk-pasangannya</t>
+          <t>1. https://motherandbeyond.id/read/28719/ide-panggilan-kakek-yang-unik-dan-kekinian-untuk-si-kecil
+2. https://motherandbeyond.id/read/28659/30-rekomendasi-nama-panggilan-tante-aesthetic-dan-kekinian
+3. https://motherandbeyond.id/read/27740/ide-panggilan-sayang-yang-unik-dan-langka-untuk-pasangan
+4. https://motherandbeyond.id/read/23681/deretan-panggilan-sayang-unik-selebriti-untuk-pasangannya</t>
         </is>
       </c>
     </row>
@@ -1004,11 +1001,11 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>1. Arti Mimpi Anak Jatuh ke Sumur tapi Selamat Menurut Primbon Jawa (AI Citation Score: 9/10 | Type: Definitional)
-2. Makna Mimpi Anak Jatuh ke Sumur dalam Pandangan Islam (AI Citation Score: 8/10 | Type: Definitional)
-3. Penjelasan Psikologis: Kecemasan Orang Tua dalam Mimpi (AI Citation Score: 8/10 | Type: Factual)
-4. Variasi Mimpi Sumur Lainnya dan Artinya (AI Citation Score: 8/10 | Type: Comparative)
-5. Yang Sebaiknya Dilakukan Setelah Mimpi Buruk tentang Anak (AI Citation Score: 7/10 | Type: Procedural)</t>
+          <t>1. Arti Mimpi Anak Jatuh ke Sumur tapi Selamat Menurut Primbon Jawa
+2. Makna Mimpi Anak Jatuh ke Sumur dalam Pandangan Islam
+3. Penjelasan Psikologis: Kecemasan Orang Tua dalam Mimpi
+4. Variasi Mimpi Sumur Lainnya dan Artinya
+5. Yang Sebaiknya Dilakukan Setelah Mimpi Buruk tentang Anak</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1025,12 +1022,12 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: arti mimpi anak tenggelam → URL: https://motherandbeyond.id/read/28057/mimpi-anak-tenggelam-apa-artinya-bagi-orang-tua
-2. Anchor: arti mimpi anak sakit → URL: https://motherandbeyond.id/read/27931/tidak-selalu-pertanda-buruk-ini-arti-mimpi-anak-sakit
-3. Anchor: arti mimpi anak meninggal → URL: https://motherandbeyond.id/read/27732/arti-mimpi-anak-meninggal-apakah-merupakan-pertanda-buruk
-4. Anchor: arti mimpi bertemu anak kecil yang tidak dikenal → URL: https://motherandbeyond.id/read/27597/arti-mimpi-bertemu-anak-kecil-yang-tidak-dikenal-adanya-kebutuhan-emosional-yang-perlu-dipenuhi
-5. Anchor: mimpi dikejar anak kecil → URL: https://motherandbeyond.id/read/27648/mimpi-dikejar-anak-kecil-apakah-pertanda-keberuntungan-atau-teguran
-6. Anchor: mimpi anak tumbuh gigi → URL: https://motherandbeyond.id/read/27800/mimpi-anak-tumbuh-gigi-pertanda-baik-atau-justru-buruk</t>
+          <t>1. https://motherandbeyond.id/read/28057/mimpi-anak-tenggelam-apa-artinya-bagi-orang-tua
+2. https://motherandbeyond.id/read/27931/tidak-selalu-pertanda-buruk-ini-arti-mimpi-anak-sakit
+3. https://motherandbeyond.id/read/27732/arti-mimpi-anak-meninggal-apakah-merupakan-pertanda-buruk
+4. https://motherandbeyond.id/read/27597/arti-mimpi-bertemu-anak-kecil-yang-tidak-dikenal-adanya-kebutuhan-emosional-yang-perlu-dipenuhi
+5. https://motherandbeyond.id/read/27648/mimpi-dikejar-anak-kecil-apakah-pertanda-keberuntungan-atau-teguran
+6. https://motherandbeyond.id/read/27800/mimpi-anak-tumbuh-gigi-pertanda-baik-atau-justru-buruk</t>
         </is>
       </c>
     </row>
@@ -1050,11 +1047,11 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>1. Arti Nama Nadia dan Asal Bahasanya (AI Citation Score: 10/10 | Type: Definitional)
-2. Makna Nama Nadia dalam Islam, Bahasa Slavia, dan Budaya Lain (AI Citation Score: 8/10 | Type: Comparative)
-3. Karakter dan Kepribadian yang Sering Dikaitkan dengan Nama Nadia (AI Citation Score: 7/10 | Type: Factual)
-4. Rangkaian Nama Nadia yang Indah: 2 Kata dan 3 Kata (AI Citation Score: 10/10 | Type: Recommendation)
-5. Tips Memadukan Nama Nadia dengan Nama Tengah dan Nama Keluarga (AI Citation Score: 7/10 | Type: Procedural)</t>
+          <t>1. Arti Nama Nadia dan Asal Bahasanya
+2. Makna Nama Nadia dalam Islam, Bahasa Slavia, dan Budaya Lain
+3. Karakter dan Kepribadian yang Sering Dikaitkan dengan Nama Nadia
+4. Rangkaian Nama Nadia yang Indah: 2 Kata dan 3 Kata
+5. Tips Memadukan Nama Nadia dengan Nama Tengah dan Nama Keluarga</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1071,12 +1068,12 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: arti nama Aluna dan rangkaiannya → URL: https://motherandbeyond.id/read/28068/arti-nama-aluna-dan-ide-rangkaian-namanya-yang-indah
-2. Anchor: arti nama Aqila → URL: https://motherandbeyond.id/read/27748/arti-nama-aqila-dan-ide-rangkaian-namanya-yang-indah
-3. Anchor: arti nama Safira → URL: https://motherandbeyond.id/read/28032/arti-nama-safira-dan-ide-rangkaian-namanya-yang-indah
-4. Anchor: arti nama Khairunnisa → URL: https://motherandbeyond.id/read/28292/arti-nama-khairunnisa-dan-ide-rangkaian-namanya-yang-indah
-5. Anchor: rangkaian nama bayi perempuan islami 2 kata → URL: https://motherandbeyond.id/read/28700/100-rangkaian-nama-bayi-perempuan-islami-2-kata-yang-cantik
-6. Anchor: nama bayi perempuan pembawa rezeki → URL: https://motherandbeyond.id/read/16493/nama-bayi-perempuan-pembawa-rezeki-dan-keberuntungan</t>
+          <t>1. https://motherandbeyond.id/read/28068/arti-nama-aluna-dan-ide-rangkaian-namanya-yang-indah
+2. https://motherandbeyond.id/read/27748/arti-nama-aqila-dan-ide-rangkaian-namanya-yang-indah
+3. https://motherandbeyond.id/read/28032/arti-nama-safira-dan-ide-rangkaian-namanya-yang-indah
+4. https://motherandbeyond.id/read/28292/arti-nama-khairunnisa-dan-ide-rangkaian-namanya-yang-indah
+5. https://motherandbeyond.id/read/28700/100-rangkaian-nama-bayi-perempuan-islami-2-kata-yang-cantik
+6. https://motherandbeyond.id/read/16493/nama-bayi-perempuan-pembawa-rezeki-dan-keberuntungan</t>
         </is>
       </c>
     </row>
@@ -1096,11 +1093,11 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>1. Pentingnya Dukungan Orang Tua bagi Anak yang Mondok di Pesantren (AI Citation Score: 7/10 | Type: Factual)
-2. Ucapan Penyemangat untuk Anak yang Sedang Menuntut Ilmu di Pesantren (AI Citation Score: 10/10 | Type: Recommendation)
-3. Ucapan Penuh Doa dan Kutipan Islami untuk Anak Santri (AI Citation Score: 9/10 | Type: Recommendation)
-4. Ucapan untuk Anak yang Baru Masuk Pesantren dan Sedang Rindu Rumah (AI Citation Score: 8/10 | Type: Recommendation)
-5. Cara Menyampaikan Pesan Lewat Surat, Kunjungan, atau Telepon Pesantren (AI Citation Score: 7/10 | Type: Procedural)</t>
+          <t>1. Pentingnya Dukungan Orang Tua bagi Anak yang Mondok di Pesantren
+2. Ucapan Penyemangat untuk Anak yang Sedang Menuntut Ilmu di Pesantren
+3. Ucapan Penuh Doa dan Kutipan Islami untuk Anak Santri
+4. Ucapan untuk Anak yang Baru Masuk Pesantren dan Sedang Rindu Rumah
+5. Cara Menyampaikan Pesan Lewat Surat, Kunjungan, atau Telepon Pesantren</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -1117,10 +1114,10 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: kata-kata doa untuk anak perempuan tersayang → URL: https://motherandbeyond.id/read/27727/50-kata-kata-doa-untuk-anak-perempuan-tersayang-agar-tumbuh-bahagia
-2. Anchor: kata-kata ibu rindu anak → URL: https://motherandbeyond.id/read/27467/50-kata-kata-ibu-rindu-anak-yang-menyentuh-dan-penuh-makna
-3. Anchor: kata-kata motivasi untuk anak SD → URL: https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
-4. Anchor: kata mutiara islami untuk anak perempuan → URL: https://motherandbeyond.id/read/17989/15-kata-mutiara-untuk-anak-perempuan-islami</t>
+          <t>1. https://motherandbeyond.id/read/27727/50-kata-kata-doa-untuk-anak-perempuan-tersayang-agar-tumbuh-bahagia
+2. https://motherandbeyond.id/read/27467/50-kata-kata-ibu-rindu-anak-yang-menyentuh-dan-penuh-makna
+3. https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
+4. https://motherandbeyond.id/read/17989/15-kata-mutiara-untuk-anak-perempuan-islami</t>
         </is>
       </c>
     </row>
@@ -1140,11 +1137,11 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>1. Arti Mimpi Melihat Anak Buang Air Besar dan Membersihkannya (AI Citation Score: 10/10 | Type: Definitional)
-2. Tafsir Mimpi Ini Menurut Islam dan Primbon Jawa (AI Citation Score: 8/10 | Type: Comparative)
-3. Makna Psikologis: Naluri Merawat dan Beban Tanggung Jawab Orang Tua (AI Citation Score: 8/10 | Type: Factual)
-4. Variasi Mimpi Buang Air Besar Lainnya dan Artinya (AI Citation Score: 8/10 | Type: Comparative)
-5. Yang Bisa Dilakukan Setelah Mengalami Mimpi Ini (AI Citation Score: 6/10 | Type: Procedural)</t>
+          <t>1. Arti Mimpi Melihat Anak Buang Air Besar dan Membersihkannya
+2. Tafsir Mimpi Ini Menurut Islam dan Primbon Jawa
+3. Makna Psikologis: Naluri Merawat dan Beban Tanggung Jawab Orang Tua
+4. Variasi Mimpi Buang Air Besar Lainnya dan Artinya
+5. Yang Bisa Dilakukan Setelah Mengalami Mimpi Ini</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
@@ -1161,12 +1158,12 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: mimpi memandikan bayi → URL: https://motherandbeyond.id/read/27673/mimpi-memandikan-bayi-benarkah-pertanda-baik
-2. Anchor: mimpi menyusui bayi sebelah kiri → URL: https://motherandbeyond.id/read/27679/mimpi-menyusui-bayi-sebelah-kiri-apa-benar-simbol-rezeki
-3. Anchor: mimpi menggendong bayi laki-laki → URL: https://motherandbeyond.id/read/27625/selain-pertanda-datangnya-rezeki-ini-7-arti-mimpi-menggendong-bayi-laki-laki
-4. Anchor: mimpi bertemu anak kecil yang tidak dikenal → URL: https://motherandbeyond.id/read/27597/arti-mimpi-bertemu-anak-kecil-yang-tidak-dikenal-adanya-kebutuhan-emosional-yang-perlu-dipenuhi
-5. Anchor: mimpi memarahi anak sendiri → URL: https://motherandbeyond.id/read/27661/mimpi-memarahi-anak-sendiri-ini-artinya-moms
-6. Anchor: frekuensi normal BAB newborn → URL: https://motherandbeyond.id/read/13363/berapa-kali-dalam-sehari-frekuensi-normal-bab-newborn</t>
+          <t>1. https://motherandbeyond.id/read/27673/mimpi-memandikan-bayi-benarkah-pertanda-baik
+2. https://motherandbeyond.id/read/27679/mimpi-menyusui-bayi-sebelah-kiri-apa-benar-simbol-rezeki
+3. https://motherandbeyond.id/read/27625/selain-pertanda-datangnya-rezeki-ini-7-arti-mimpi-menggendong-bayi-laki-laki
+4. https://motherandbeyond.id/read/27597/arti-mimpi-bertemu-anak-kecil-yang-tidak-dikenal-adanya-kebutuhan-emosional-yang-perlu-dipenuhi
+5. https://motherandbeyond.id/read/27661/mimpi-memarahi-anak-sendiri-ini-artinya-moms
+6. https://motherandbeyond.id/read/13363/berapa-kali-dalam-sehari-frekuensi-normal-bab-newborn</t>
         </is>
       </c>
     </row>
@@ -1186,11 +1183,11 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>1. Tips Memilih Kado Sesuai Minat dan Tahap Perkembangan Anak 7 Tahun (AI Citation Score: 8/10 | Type: Procedural)
-2. Rekomendasi Kado Kreatif dan Edukatif untuk Anak Perempuan 7 Tahun (AI Citation Score: 10/10 | Type: Recommendation)
-3. Ide Kado Perlengkapan Sekolah dan Dekorasi Kamar yang Disukai Anak (AI Citation Score: 8/10 | Type: Recommendation)
-4. Kado Murah Meriah di Bawah Rp100 Ribu (AI Citation Score: 9/10 | Type: Recommendation)
-5. Tabel Perbandingan Kado: Manfaat, Kisaran Harga, dan Cocok untuk Siapa (AI Citation Score: 8/10 | Type: Comparative)</t>
+          <t>1. Tips Memilih Kado Sesuai Minat dan Tahap Perkembangan Anak 7 Tahun
+2. Rekomendasi Kado Kreatif dan Edukatif untuk Anak Perempuan 7 Tahun
+3. Ide Kado Perlengkapan Sekolah dan Dekorasi Kamar yang Disukai Anak
+4. Kado Murah Meriah di Bawah Rp100 Ribu
+5. Tabel Perbandingan Kado: Manfaat, Kisaran Harga, dan Cocok untuk Siapa</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -1207,10 +1204,10 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: kado untuk anak laki-laki 4 tahun → URL: https://motherandbeyond.id/read/26685/bingung-cari-kado-untuk-anak-laki-laki-4-tahun-ini-pilihan-terbaiknya
-2. Anchor: kata-kata doa untuk anak perempuan tersayang → URL: https://motherandbeyond.id/read/27727/50-kata-kata-doa-untuk-anak-perempuan-tersayang-agar-tumbuh-bahagia
-3. Anchor: kado bayi yang bermanfaat jangka panjang → URL: https://motherandbeyond.id/read/27898/10-kado-bayi-yang-bermanfaat-untuk-jangka-panjang-sampai-ia-besar
-4. Anchor: manfaat pop it fidget toy → URL: https://motherandbeyond.id/read/23087/bukan-mainan-biasa-ini-manfaat-dari-pop-it-fidget-toy-buat-anak</t>
+          <t>1. https://motherandbeyond.id/read/26685/bingung-cari-kado-untuk-anak-laki-laki-4-tahun-ini-pilihan-terbaiknya
+2. https://motherandbeyond.id/read/27727/50-kata-kata-doa-untuk-anak-perempuan-tersayang-agar-tumbuh-bahagia
+3. https://motherandbeyond.id/read/27898/10-kado-bayi-yang-bermanfaat-untuk-jangka-panjang-sampai-ia-besar
+4. https://motherandbeyond.id/read/23087/bukan-mainan-biasa-ini-manfaat-dari-pop-it-fidget-toy-buat-anak</t>
         </is>
       </c>
     </row>
@@ -1230,11 +1227,11 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Sekolah Inklusi dan Bedanya dengan SLB? (AI Citation Score: 10/10 | Type: Definitional)
-2. Daftar Sekolah Inklusi di Jakarta Negeri dan Swasta (AI Citation Score: 10/10 | Type: Recommendation)
-3. Perkiraan Biaya Sekolah Inklusi di Jakarta (AI Citation Score: 9/10 | Type: Factual)
-4. Cara Memilih Sekolah Inklusi yang Tepat untuk Anak Berkebutuhan Khusus (AI Citation Score: 9/10 | Type: Procedural)
-5. Alur Pendaftaran dan Dokumen yang Perlu Disiapkan (AI Citation Score: 8/10 | Type: Procedural)</t>
+          <t>1. Apa Itu Sekolah Inklusi dan Bedanya dengan SLB?
+2. Daftar Sekolah Inklusi di Jakarta Negeri dan Swasta
+3. Perkiraan Biaya Sekolah Inklusi di Jakarta
+4. Cara Memilih Sekolah Inklusi yang Tepat untuk Anak Berkebutuhan Khusus
+5. Alur Pendaftaran dan Dokumen yang Perlu Disiapkan</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
@@ -1251,10 +1248,9 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: perbedaan autis dan down syndrome → URL: https://motherandbeyond.id/read/28660/perbedaan-autis-dan-down-syndrome-yang-perlu-diketahui
-2. Anchor: ciri anak hiperaktif → URL: https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun
-3. Anchor: cara menghitung tahun lulus sekolah anak → URL: https://motherandbeyond.id/read/27879/begini-cara-menghitung-tahun-lulus-sekolah-anak-tanpa-pusing
-Limited relevant internal link available from Ahrefs export.</t>
+          <t>1. https://motherandbeyond.id/read/28660/perbedaan-autis-dan-down-syndrome-yang-perlu-diketahui
+2. https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun
+3. https://motherandbeyond.id/read/27879/begini-cara-menghitung-tahun-lulus-sekolah-anak-tanpa-pusing</t>
         </is>
       </c>
     </row>
@@ -1274,11 +1270,11 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Overstimulasi pada Ibu? (AI Citation Score: 10/10 | Type: Definitional)
-2. Penyebab Ibu Mudah Overstimulasi: Sensory Overload dan Mental Load (AI Citation Score: 9/10 | Type: Factual)
-3. Ciri-Ciri Overstimulasi yang Sering Tidak Disadari Ibu (AI Citation Score: 10/10 | Type: Factual)
-4. Overstimulasi, Burnout, atau Baby Blues? Kenali Bedanya (AI Citation Score: 9/10 | Type: Comparative)
-5. Cara Mengatasi Overstimulasi dan Kapan Perlu Bantuan Profesional (AI Citation Score: 9/10 | Type: Procedural)</t>
+          <t>1. Apa Itu Overstimulasi pada Ibu?
+2. Penyebab Ibu Mudah Overstimulasi: Sensory Overload dan Mental Load
+3. Ciri-Ciri Overstimulasi yang Sering Tidak Disadari Ibu
+4. Overstimulasi, Burnout, atau Baby Blues? Kenali Bedanya
+5. Cara Mengatasi Overstimulasi dan Kapan Perlu Bantuan Profesional</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -1295,10 +1291,10 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: manfaat hidup rukun dalam keluarga untuk mengurangi stres → URL: https://motherandbeyond.id/read/25369/6-manfaat-hidup-rukun-dalam-keluarga-bisa-mengurangi-stres
-2. Anchor: penyebab badan sakit semua pada wanita → URL: https://motherandbeyond.id/read/27549/9-penyebab-badan-sakit-semua-pada-wanita-dan-cara-mengatasinya
-3. Anchor: pantangan ibu baru melahirkan sebelum 40 hari → URL: https://motherandbeyond.id/read/26873/pantangan-ibu-baru-melahirkan-sebelum-40-hari-mitos-atau-fakta-medis
-4. Anchor: balita cengeng dan cara mengatasinya → URL: https://motherandbeyond.id/read/17263/balita-cengeng-ini-penyebab-dan-cara-mengatasinya</t>
+          <t>1. https://motherandbeyond.id/read/25369/6-manfaat-hidup-rukun-dalam-keluarga-bisa-mengurangi-stres
+2. https://motherandbeyond.id/read/27549/9-penyebab-badan-sakit-semua-pada-wanita-dan-cara-mengatasinya
+3. https://motherandbeyond.id/read/26873/pantangan-ibu-baru-melahirkan-sebelum-40-hari-mitos-atau-fakta-medis
+4. https://motherandbeyond.id/read/17263/balita-cengeng-ini-penyebab-dan-cara-mengatasinya</t>
         </is>
       </c>
     </row>
@@ -1318,11 +1314,11 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>1. Mengapa Anak Takut Menghadapi Ujian Sekolah? (AI Citation Score: 9/10 | Type: Factual)
-2. Mengenal Test Anxiety: Ciri-Ciri Kecemasan Ujian pada Anak (AI Citation Score: 10/10 | Type: Definitional)
-3. Cemas Ujian yang Wajar vs yang Perlu Diwaspadai (AI Citation Score: 8/10 | Type: Comparative)
-4. Cara Membantu Anak Mengatasi Takut Ujian Sebelum dan Saat Hari-H (AI Citation Score: 10/10 | Type: Procedural)
-5. Peran Orang Tua: Kalimat yang Sebaiknya Diucapkan dan Dihindari (AI Citation Score: 8/10 | Type: Recommendation)</t>
+          <t>1. Mengapa Anak Takut Menghadapi Ujian Sekolah?
+2. Mengenal Test Anxiety: Ciri-Ciri Kecemasan Ujian pada Anak
+3. Cemas Ujian yang Wajar vs yang Perlu Diwaspadai
+4. Cara Membantu Anak Mengatasi Takut Ujian Sebelum dan Saat Hari-H
+5. Peran Orang Tua: Kalimat yang Sebaiknya Diucapkan dan Dihindari</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
@@ -1339,11 +1335,11 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: kata-kata motivasi untuk anak SD → URL: https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
-2. Anchor: 100 soal pengetahuan umum SD → URL: https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
-3. Anchor: ide menu bekal sekolah anak SD → URL: https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi
-4. Anchor: anak batuk psikogenik → URL: https://motherandbeyond.id/read/11721/anak-batuk-psikogenik-ini-penyebab-dan-cara-mengatasi
-5. Anchor: kata-kata motivasi untuk keluarga → URL: https://motherandbeyond.id/read/27023/70-kata-kata-motivasi-untuk-keluarga-yang-menginspirasi</t>
+          <t>1. https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
+2. https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
+3. https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi
+4. https://motherandbeyond.id/read/11721/anak-batuk-psikogenik-ini-penyebab-dan-cara-mengatasi
+5. https://motherandbeyond.id/read/27023/70-kata-kata-motivasi-untuk-keluarga-yang-menginspirasi</t>
         </is>
       </c>
     </row>
@@ -1363,11 +1359,11 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Influenza A pada Anak dan Bedanya dengan Flu Biasa? (AI Citation Score: 10/10 | Type: Definitional)
-2. Gejala Influenza A pada Anak yang Perlu Dikenali (AI Citation Score: 10/10 | Type: Factual)
-3. Tanda Bahaya Influenza A: Kapan Anak Harus Dibawa ke Dokter atau IGD? (AI Citation Score: 10/10 | Type: Procedural)
-4. Cara Merawat Anak dengan Influenza A di Rumah (AI Citation Score: 9/10 | Type: Procedural)
-5. Cara Mencegah Influenza A: Vaksin Flu dan Kebiasaan Sehat (AI Citation Score: 9/10 | Type: Factual)</t>
+          <t>1. Apa Itu Influenza A pada Anak dan Bedanya dengan Flu Biasa?
+2. Gejala Influenza A pada Anak yang Perlu Dikenali
+3. Tanda Bahaya Influenza A: Kapan Anak Harus Dibawa ke Dokter atau IGD?
+4. Cara Merawat Anak dengan Influenza A di Rumah
+5. Cara Mencegah Influenza A: Vaksin Flu dan Kebiasaan Sehat</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -1384,12 +1380,12 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: obat tradisional batuk pilek untuk bayi 0-6 bulan → URL: https://motherandbeyond.id/read/26882/obat-tradisional-batuk-pilek-untuk-bayi-0-6-bulan-yang-aman-dan-alami
-2. Anchor: anak demam tapi tangan dan kaki dingin → URL: https://motherandbeyond.id/read/26753/5-cara-mengatasi-anak-demam-tapi-tangan-dan-kaki-dingin
-3. Anchor: demam anak naik turun selama 3 hari → URL: https://motherandbeyond.id/read/27685/demam-anak-naik-turun-selama-3-hari-ini-penyebab-dan-cara-penanganannya
-4. Anchor: cara tepat mengukur suhu anak demam → URL: https://motherandbeyond.id/read/5105/cara-tepat-ukur-suhu-anak-demam
-5. Anchor: kejang demam pada bayi → URL: https://motherandbeyond.id/read/22211/kejang-demam-pada-bayi-ini-yang-perlu-anda-perhatikan
-6. Anchor: makanan dan minuman yang bantu turunkan demam anak → URL: https://motherandbeyond.id/read/17871/7-makanan-dan-minuman-yang-bantu-turunkan-demam-anak</t>
+          <t>1. https://motherandbeyond.id/read/26882/obat-tradisional-batuk-pilek-untuk-bayi-0-6-bulan-yang-aman-dan-alami
+2. https://motherandbeyond.id/read/26753/5-cara-mengatasi-anak-demam-tapi-tangan-dan-kaki-dingin
+3. https://motherandbeyond.id/read/27685/demam-anak-naik-turun-selama-3-hari-ini-penyebab-dan-cara-penanganannya
+4. https://motherandbeyond.id/read/5105/cara-tepat-ukur-suhu-anak-demam
+5. https://motherandbeyond.id/read/22211/kejang-demam-pada-bayi-ini-yang-perlu-anda-perhatikan
+6. https://motherandbeyond.id/read/17871/7-makanan-dan-minuman-yang-bantu-turunkan-demam-anak</t>
         </is>
       </c>
     </row>
@@ -1409,11 +1405,11 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>1. Kenapa Anak Mudah Menyerah Saat Belajar? (AI Citation Score: 9/10 | Type: Factual)
-2. Mengenal Grit dan Growth Mindset pada Anak (AI Citation Score: 9/10 | Type: Definitional)
-3. Mudah Menyerah Biasa atau Tanda Masalah Konsentrasi dan Belajar? (AI Citation Score: 8/10 | Type: Comparative)
-4. Cara Melatih Anak agar Tidak Mudah Menyerah Saat Belajar (AI Citation Score: 10/10 | Type: Procedural)
-5. Contoh Kalimat Pujian yang Membangun Daya Juang Anak (AI Citation Score: 8/10 | Type: Recommendation)</t>
+          <t>1. Kenapa Anak Mudah Menyerah Saat Belajar?
+2. Mengenal Grit dan Growth Mindset pada Anak
+3. Mudah Menyerah Biasa atau Tanda Masalah Konsentrasi dan Belajar?
+4. Cara Melatih Anak agar Tidak Mudah Menyerah Saat Belajar
+5. Contoh Kalimat Pujian yang Membangun Daya Juang Anak</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -1430,10 +1426,10 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: kata-kata motivasi untuk anak SD → URL: https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
-2. Anchor: ciri anak hiperaktif → URL: https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun
-3. Anchor: balita cengeng dan cara mengatasinya → URL: https://motherandbeyond.id/read/17263/balita-cengeng-ini-penyebab-dan-cara-mengatasinya
-4. Anchor: cara mengatasi balita yang suka melawan orang tua → URL: https://motherandbeyond.id/read/20609/cara-tepat-mengatasi-balita-yang-suka-melawan-orang-tua</t>
+          <t>1. https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
+2. https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun
+3. https://motherandbeyond.id/read/17263/balita-cengeng-ini-penyebab-dan-cara-mengatasinya
+4. https://motherandbeyond.id/read/20609/cara-tepat-mengatasi-balita-yang-suka-melawan-orang-tua</t>
         </is>
       </c>
     </row>
@@ -1453,11 +1449,11 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>1. Seperti Apa Gerakan Janin Menjelang Persalinan? (AI Citation Score: 10/10 | Type: Definitional)
-2. Perubahan Pola Gerakan Janin di Trimester Akhir: Lebih Kuat, Menggeliat, dan Terasa di Bawah (AI Citation Score: 9/10 | Type: Factual)
-3. Gerakan Janin Normal vs Berkurang: Kapan Harus Waspada? (AI Citation Score: 10/10 | Type: Comparative)
-4. Cara Menghitung Gerakan Janin di Rumah (Metode Hitung 10) (AI Citation Score: 9/10 | Type: Procedural)
-5. Tanda Persalinan Lain yang Muncul Bersamaan dengan Perubahan Gerakan Janin (AI Citation Score: 8/10 | Type: Factual)</t>
+          <t>1. Seperti Apa Gerakan Janin Menjelang Persalinan?
+2. Perubahan Pola Gerakan Janin di Trimester Akhir: Lebih Kuat, Menggeliat, dan Terasa di Bawah
+3. Gerakan Janin Normal vs Berkurang: Kapan Harus Waspada?
+4. Cara Menghitung Gerakan Janin di Rumah (Metode Hitung 10)
+5. Tanda Persalinan Lain yang Muncul Bersamaan dengan Perubahan Gerakan Janin</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -1474,12 +1470,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: ciri-ciri janin masuk panggul → URL: https://motherandbeyond.id/read/27640/ini-ciri-ciri-janin-masuk-panggul-yang-perlu-ibu-hamil-kenali
-2. Anchor: ciri akan melahirkan dalam 2 minggu lagi → URL: https://motherandbeyond.id/read/26813/kenali-ciri-ciri-anda-akan-melahirkan-dalam-2-minggu-lagi
-3. Anchor: tanda melahirkan pembukaan 1 → URL: https://motherandbeyond.id/read/25437/7-tanda-melahirkan-pembukaan-1-yang-perlu-moms-kenali
-4. Anchor: ciri air ketuban merembes → URL: https://motherandbeyond.id/read/24069/air-ketuban-merembes-ini-ciri-cirinya-yang-perlu-anda-kenali
-5. Anchor: janin terlalu aktif bergerak → URL: https://motherandbeyond.id/read/18795/janin-terlalu-aktif-bergerak-ini-penyebabnya-moms
-6. Anchor: cara mengatasi kontraksi palsu saat hamil 8 bulan → URL: https://motherandbeyond.id/read/27798/cara-mengatasi-kontraksi-palsu-saat-hamil-8-bulan</t>
+          <t>1. https://motherandbeyond.id/read/27640/ini-ciri-ciri-janin-masuk-panggul-yang-perlu-ibu-hamil-kenali
+2. https://motherandbeyond.id/read/26813/kenali-ciri-ciri-anda-akan-melahirkan-dalam-2-minggu-lagi
+3. https://motherandbeyond.id/read/25437/7-tanda-melahirkan-pembukaan-1-yang-perlu-moms-kenali
+4. https://motherandbeyond.id/read/24069/air-ketuban-merembes-ini-ciri-cirinya-yang-perlu-anda-kenali
+5. https://motherandbeyond.id/read/18795/janin-terlalu-aktif-bergerak-ini-penyebabnya-moms
+6. https://motherandbeyond.id/read/27798/cara-mengatasi-kontraksi-palsu-saat-hamil-8-bulan</t>
         </is>
       </c>
     </row>
@@ -1499,11 +1495,11 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Numerasi pada Anak dan Bedanya dengan Matematika? (AI Citation Score: 10/10 | Type: Definitional)
-2. Aspek Numerasi Anak: Berhitung, Relasi Bilangan, dan Operasi Dasar (AI Citation Score: 9/10 | Type: Factual)
-3. Tahapan Kemampuan Numerasi Anak Sesuai Usia (AI Citation Score: 9/10 | Type: Factual)
-4. Cara Mengenalkan Numerasi pada Anak di Rumah Lewat Bermain (AI Citation Score: 10/10 | Type: Procedural)
-5. Ide Aktivitas dan Permainan Numerasi Sehari-hari (AI Citation Score: 8/10 | Type: Recommendation)</t>
+          <t>1. Apa Itu Numerasi pada Anak dan Bedanya dengan Matematika?
+2. Aspek Numerasi Anak: Berhitung, Relasi Bilangan, dan Operasi Dasar
+3. Tahapan Kemampuan Numerasi Anak Sesuai Usia
+4. Cara Mengenalkan Numerasi pada Anak di Rumah Lewat Bermain
+5. Ide Aktivitas dan Permainan Numerasi Sehari-hari</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
@@ -1520,10 +1516,9 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: 100 soal pengetahuan umum SD → URL: https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
-2. Anchor: mainan bayi 5 bulan untuk tumbuh kembang → URL: https://motherandbeyond.id/read/27315/mainan-bayi-5-bulan-untuk-dukung-tumbuh-kembangnya
-3. Anchor: dongeng sebelum tidur yang singkat → URL: https://motherandbeyond.id/read/25388/dongeng-sebelum-tidur-yang-singkat-dan-penuh-makna-untuk-anak
-Limited relevant internal link available from Ahrefs export.</t>
+          <t>1. https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
+2. https://motherandbeyond.id/read/27315/mainan-bayi-5-bulan-untuk-dukung-tumbuh-kembangnya
+3. https://motherandbeyond.id/read/25388/dongeng-sebelum-tidur-yang-singkat-dan-penuh-makna-untuk-anak</t>
         </is>
       </c>
     </row>
@@ -1543,11 +1538,11 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Potongan Rambut Mangkok (Bowl Cut) untuk Anak? (AI Citation Score: 9/10 | Type: Definitional)
-2. Model Rambut Mangkok Anak yang Populer: Klasik, Fringe, hingga Undercut (AI Citation Score: 10/10 | Type: Recommendation)
-3. Rambut Mangkok Cocok untuk Bentuk Wajah dan Jenis Rambut Seperti Apa? (AI Citation Score: 8/10 | Type: Comparative)
-4. Cara Memotong Rambut Mangkok Anak Sendiri di Rumah (AI Citation Score: 9/10 | Type: Procedural)
-5. Tips Merawat Rambut Mangkok Anak agar Tetap Rapi (AI Citation Score: 7/10 | Type: Procedural)</t>
+          <t>1. Apa Itu Potongan Rambut Mangkok (Bowl Cut) untuk Anak?
+2. Model Rambut Mangkok Anak yang Populer: Klasik, Fringe, hingga Undercut
+3. Rambut Mangkok Cocok untuk Bentuk Wajah dan Jenis Rambut Seperti Apa?
+4. Cara Memotong Rambut Mangkok Anak Sendiri di Rumah
+5. Tips Merawat Rambut Mangkok Anak agar Tetap Rapi</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
@@ -1564,10 +1559,9 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: model rambut anak cowok terbaru → URL: https://motherandbeyond.id/read/28709/15-model-rambut-anak-cowok-terbaru-rapi-keren-dan-sesuai-aturan-sekolah
-2. Anchor: potongan rambut buzz cut anak → URL: https://motherandbeyond.id/read/28651/potongan-rambut-buzz-cut-anak-untuk-si-kecil-yang-aktif
-3. Anchor: trik agar anak mau potong rambut → URL: https://motherandbeyond.id/read/12131/7-trik-agar-anak-mau-potong-rambut
-Limited relevant internal link available from Ahrefs export.</t>
+          <t>1. https://motherandbeyond.id/read/28709/15-model-rambut-anak-cowok-terbaru-rapi-keren-dan-sesuai-aturan-sekolah
+2. https://motherandbeyond.id/read/28651/potongan-rambut-buzz-cut-anak-untuk-si-kecil-yang-aktif
+3. https://motherandbeyond.id/read/12131/7-trik-agar-anak-mau-potong-rambut</t>
         </is>
       </c>
     </row>
@@ -1587,11 +1581,11 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu PAUD dan TK? Pengertian Singkatnya (AI Citation Score: 10/10 | Type: Definitional)
-2. Perbedaan PAUD dan TK: Usia, Jalur Pendidikan, dan Kurikulum (AI Citation Score: 10/10 | Type: Comparative)
-3. Jenis-Jenis Satuan PAUD: KB, TPA, SPS, hingga TK/RA (AI Citation Score: 8/10 | Type: Factual)
-4. Apakah Anak Wajib PAUD atau TK Sebelum Masuk SD? (AI Citation Score: 9/10 | Type: Factual)
-5. Cara Memilih PAUD atau TK yang Sesuai dengan Usia dan Kebutuhan Anak (AI Citation Score: 8/10 | Type: Procedural)</t>
+          <t>1. Apa Itu PAUD dan TK? Pengertian Singkatnya
+2. Perbedaan PAUD dan TK: Usia, Jalur Pendidikan, dan Kurikulum
+3. Jenis-Jenis Satuan PAUD: KB, TPA, SPS, hingga TK/RA
+4. Apakah Anak Wajib PAUD atau TK Sebelum Masuk SD?
+5. Cara Memilih PAUD atau TK yang Sesuai dengan Usia dan Kebutuhan Anak</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
@@ -1608,10 +1602,10 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: cara menghitung tahun lulus sekolah anak → URL: https://motherandbeyond.id/read/27879/begini-cara-menghitung-tahun-lulus-sekolah-anak-tanpa-pusing
-2. Anchor: ide menu bekal sekolah anak → URL: https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi
-3. Anchor: dongeng sebelum tidur yang singkat → URL: https://motherandbeyond.id/read/25388/dongeng-sebelum-tidur-yang-singkat-dan-penuh-makna-untuk-anak
-4. Anchor: ciri anak hiperaktif → URL: https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun</t>
+          <t>1. https://motherandbeyond.id/read/27879/begini-cara-menghitung-tahun-lulus-sekolah-anak-tanpa-pusing
+2. https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi
+3. https://motherandbeyond.id/read/25388/dongeng-sebelum-tidur-yang-singkat-dan-penuh-makna-untuk-anak
+4. https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun</t>
         </is>
       </c>
     </row>
@@ -1631,11 +1625,11 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>1. Arti Mimpi Punya Adik Perempuan Secara Umum (AI Citation Score: 10/10 | Type: Definitional)
-2. Tafsir Mimpi Punya Adik Perempuan Menurut Islam dan Primbon Jawa (AI Citation Score: 8/10 | Type: Comparative)
-3. Makna Psikologis: Kebutuhan Kasih Sayang dan Tanggung Jawab Baru (AI Citation Score: 8/10 | Type: Factual)
-4. Variasi Mimpi Punya Adik Perempuan dan Artinya (AI Citation Score: 9/10 | Type: Comparative)
-5. Cara Menyikapi Mimpi Ini dengan Bijak (AI Citation Score: 6/10 | Type: Procedural)</t>
+          <t>1. Arti Mimpi Punya Adik Perempuan Secara Umum
+2. Tafsir Mimpi Punya Adik Perempuan Menurut Islam dan Primbon Jawa
+3. Makna Psikologis: Kebutuhan Kasih Sayang dan Tanggung Jawab Baru
+4. Variasi Mimpi Punya Adik Perempuan dan Artinya
+5. Cara Menyikapi Mimpi Ini dengan Bijak</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
@@ -1652,12 +1646,12 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: arti mimpi punya anak perempuan → URL: https://motherandbeyond.id/read/24267/bisa-jadi-pertanda-baik-ini-6-arti-mimpi-punya-anak-perempuan
-2. Anchor: mimpi dikasih anak perempuan → URL: https://motherandbeyond.id/read/27771/mimpi-dikasih-anak-perempuan-ini-artinya-menurut-islam-dan-primbon
-3. Anchor: mimpi menggendong bayi perempuan → URL: https://motherandbeyond.id/read/28425/mimpi-menggendong-anak-bayi-perempuan-ini-maknanya
-4. Anchor: mimpi saudara menikah → URL: https://motherandbeyond.id/read/28404/mimpi-saudara-menikah-apa-maknanya-dalam-berbagai-tafsir
-5. Anchor: mimpi adik meninggal → URL: https://motherandbeyond.id/read/28441/mimpi-adik-meninggal-ini-arti-dan-cara-menyikapinya
-6. Anchor: mimpi melihat orang hamil → URL: https://motherandbeyond.id/read/26879/7-arti-mimpi-melihat-orang-hamil</t>
+          <t>1. https://motherandbeyond.id/read/24267/bisa-jadi-pertanda-baik-ini-6-arti-mimpi-punya-anak-perempuan
+2. https://motherandbeyond.id/read/27771/mimpi-dikasih-anak-perempuan-ini-artinya-menurut-islam-dan-primbon
+3. https://motherandbeyond.id/read/28425/mimpi-menggendong-anak-bayi-perempuan-ini-maknanya
+4. https://motherandbeyond.id/read/28404/mimpi-saudara-menikah-apa-maknanya-dalam-berbagai-tafsir
+5. https://motherandbeyond.id/read/28441/mimpi-adik-meninggal-ini-arti-dan-cara-menyikapinya
+6. https://motherandbeyond.id/read/26879/7-arti-mimpi-melihat-orang-hamil</t>
         </is>
       </c>
     </row>
@@ -1677,11 +1671,11 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Sekolah Negeri dan Sekolah Swasta? (AI Citation Score: 9/10 | Type: Definitional)
-2. Perbedaan Sekolah Negeri dan Swasta: Biaya, Fasilitas, Kurikulum, dan Jumlah Siswa (AI Citation Score: 10/10 | Type: Comparative)
-3. Kelebihan dan Kekurangan Sekolah Negeri (AI Citation Score: 8/10 | Type: Comparative)
-4. Kelebihan dan Kekurangan Sekolah Swasta (AI Citation Score: 8/10 | Type: Comparative)
-5. Cara Memilih Sekolah Negeri atau Swasta Sesuai Kebutuhan Anak dan Budget Keluarga (AI Citation Score: 9/10 | Type: Procedural)</t>
+          <t>1. Apa Itu Sekolah Negeri dan Sekolah Swasta?
+2. Perbedaan Sekolah Negeri dan Swasta: Biaya, Fasilitas, Kurikulum, dan Jumlah Siswa
+3. Kelebihan dan Kekurangan Sekolah Negeri
+4. Kelebihan dan Kekurangan Sekolah Swasta
+5. Cara Memilih Sekolah Negeri atau Swasta Sesuai Kebutuhan Anak dan Budget Keluarga</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
@@ -1698,10 +1692,10 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: soal pengetahuan umum SD dan jawabannya → URL: https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
-2. Anchor: cara menghitung tahun lulus sekolah anak → URL: https://motherandbeyond.id/read/27879/begini-cara-menghitung-tahun-lulus-sekolah-anak-tanpa-pusing
-3. Anchor: model rambut anak cowok sesuai aturan sekolah → URL: https://motherandbeyond.id/read/28709/15-model-rambut-anak-cowok-terbaru-rapi-keren-dan-sesuai-aturan-sekolah
-4. Anchor: ide menu bekal sekolah anak SD → URL: https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi</t>
+          <t>1. https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
+2. https://motherandbeyond.id/read/27879/begini-cara-menghitung-tahun-lulus-sekolah-anak-tanpa-pusing
+3. https://motherandbeyond.id/read/28709/15-model-rambut-anak-cowok-terbaru-rapi-keren-dan-sesuai-aturan-sekolah
+4. https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi</t>
         </is>
       </c>
     </row>
@@ -1721,11 +1715,11 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>1. Kenapa Jajanan Jadul SD Selalu Bikin Nostalgia? (AI Citation Score: 7/10 | Type: Factual)
-2. Daftar Jajanan Jadul SD Era 90-an yang Legendaris (AI Citation Score: 10/10 | Type: Recommendation)
-3. Jajanan SD Tahun 2000-an yang Masih Diingat Sampai Sekarang (AI Citation Score: 9/10 | Type: Recommendation)
-4. Jajanan Jadul SD yang Masih Bisa Ditemukan dan Dibeli Saat Ini (AI Citation Score: 8/10 | Type: Recommendation)
-5. Resep Jajanan Jadul SD yang Bisa Dibuat di Rumah Bersama Anak (AI Citation Score: 8/10 | Type: Procedural)</t>
+          <t>1. Kenapa Jajanan Jadul SD Selalu Bikin Nostalgia?
+2. Daftar Jajanan Jadul SD Era 90-an yang Legendaris
+3. Jajanan SD Tahun 2000-an yang Masih Diingat Sampai Sekarang
+4. Jajanan Jadul SD yang Masih Bisa Ditemukan dan Dibeli Saat Ini
+5. Resep Jajanan Jadul SD yang Bisa Dibuat di Rumah Bersama Anak</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
@@ -1742,10 +1736,9 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: ide menu bekal sekolah anak SD → URL: https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi
-2. Anchor: ide bekal menu 4 sehat 5 sempurna untuk anak SD → URL: https://motherandbeyond.id/read/28428/ide-bekal-dengan-menu-4-sehat-5-sempurna-untuk-anak-sd
-3. Anchor: 100 soal pengetahuan umum SD → URL: https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
-Limited relevant internal link available from Ahrefs export.</t>
+          <t>1. https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi
+2. https://motherandbeyond.id/read/28428/ide-bekal-dengan-menu-4-sehat-5-sempurna-untuk-anak-sd
+3. https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas</t>
         </is>
       </c>
     </row>
@@ -1765,11 +1758,11 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Kelahiran Sungsang Secara Medis? (AI Citation Score: 9/10 | Type: Definitional)
-2. Watak Anak yang Lahir Sungsang Menurut Kepercayaan Jawa dan Sunda (AI Citation Score: 9/10 | Type: Factual)
-3. Mitos vs Fakta: Apakah Posisi Lahir Memengaruhi Kepribadian Anak? (AI Citation Score: 10/10 | Type: Comparative)
-4. Yang Lebih Berpengaruh pada Watak Anak: Pola Asuh dan Lingkungan (AI Citation Score: 8/10 | Type: Factual)
-5. Perhatian Khusus Kesehatan untuk Bayi yang Lahir Sungsang (AI Citation Score: 8/10 | Type: Procedural)</t>
+          <t>1. Apa Itu Kelahiran Sungsang Secara Medis?
+2. Watak Anak yang Lahir Sungsang Menurut Kepercayaan Jawa dan Sunda
+3. Mitos vs Fakta: Apakah Posisi Lahir Memengaruhi Kepribadian Anak?
+4. Yang Lebih Berpengaruh pada Watak Anak: Pola Asuh dan Lingkungan
+5. Perhatian Khusus Kesehatan untuk Bayi yang Lahir Sungsang</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
@@ -1786,10 +1779,10 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: ciri-ciri janin masuk panggul → URL: https://motherandbeyond.id/read/27640/ini-ciri-ciri-janin-masuk-panggul-yang-perlu-ibu-hamil-kenali
-2. Anchor: 4 posisi janin dalam kandungan → URL: https://motherandbeyond.id/read/12686/bumil-perlu-tahu-ini-4-posisi-janin-dalam-kandungan
-3. Anchor: gentle birth, persalinan yang tenang → URL: https://motherandbeyond.id/read/12539/gentle-birth-pilihan-persalinan-yang-tenang-dan-nyaman
-4. Anchor: arti haid menurut primbon Jawa → URL: https://motherandbeyond.id/read/27723/arti-haid-menurut-hari-tanggal-dan-jam-dalam-primbon-jawa</t>
+          <t>1. https://motherandbeyond.id/read/27640/ini-ciri-ciri-janin-masuk-panggul-yang-perlu-ibu-hamil-kenali
+2. https://motherandbeyond.id/read/12686/bumil-perlu-tahu-ini-4-posisi-janin-dalam-kandungan
+3. https://motherandbeyond.id/read/12539/gentle-birth-pilihan-persalinan-yang-tenang-dan-nyaman
+4. https://motherandbeyond.id/read/27723/arti-haid-menurut-hari-tanggal-dan-jam-dalam-primbon-jawa</t>
         </is>
       </c>
     </row>
@@ -1809,11 +1802,11 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Maksud Anak Terakhir Ketemu Anak Terakhir? (AI Citation Score: 8/10 | Type: Definitional)
-2. Karakter Anak Bungsu Menurut Teori Urutan Kelahiran (AI Citation Score: 9/10 | Type: Factual)
-3. Kelebihan dan Tantangan Pasangan Sesama Anak Terakhir (AI Citation Score: 10/10 | Type: Comparative)
-4. Mitos Pernikahan Anak Terakhir dengan Anak Terakhir dalam Adat Jawa (AI Citation Score: 8/10 | Type: Factual)
-5. Tips Membangun Rumah Tangga Harmonis Sesama Anak Bungsu (AI Citation Score: 9/10 | Type: Procedural)</t>
+          <t>1. Apa Maksud Anak Terakhir Ketemu Anak Terakhir?
+2. Karakter Anak Bungsu Menurut Teori Urutan Kelahiran
+3. Kelebihan dan Tantangan Pasangan Sesama Anak Terakhir
+4. Mitos Pernikahan Anak Terakhir dengan Anak Terakhir dalam Adat Jawa
+5. Tips Membangun Rumah Tangga Harmonis Sesama Anak Bungsu</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
@@ -1830,11 +1823,11 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: fakta anak kedua menikah dengan anak kedua → URL: https://motherandbeyond.id/read/27494/jodoh-idaman-ini-fakta-anak-kedua-menikah-dengan-anak-kedua
-2. Anchor: weton ketemu 25 → URL: https://motherandbeyond.id/read/28495/weton-ketemu-25-ini-arti-tafsir-dan-cara-menyikapinya
-3. Anchor: ramalan jodoh berdasarkan tanggal lahir → URL: https://motherandbeyond.id/read/28320/ramalan-jodoh-berdasarkan-tanggal-lahir-dengan-prinsip-numerologi
-4. Anchor: ciri-ciri pasangan setia → URL: https://motherandbeyond.id/read/26256/6-ciri-ciri-pasangan-setia-yang-bisa-anda-kenali
-5. Anchor: pertanyaan truth or dare untuk pasangan → URL: https://motherandbeyond.id/read/28282/50-pertanyaan-truth-or-dare-pasangan-untuk-hubungan-makin-hangat</t>
+          <t>1. https://motherandbeyond.id/read/27494/jodoh-idaman-ini-fakta-anak-kedua-menikah-dengan-anak-kedua
+2. https://motherandbeyond.id/read/28495/weton-ketemu-25-ini-arti-tafsir-dan-cara-menyikapinya
+3. https://motherandbeyond.id/read/28320/ramalan-jodoh-berdasarkan-tanggal-lahir-dengan-prinsip-numerologi
+4. https://motherandbeyond.id/read/26256/6-ciri-ciri-pasangan-setia-yang-bisa-anda-kenali
+5. https://motherandbeyond.id/read/28282/50-pertanyaan-truth-or-dare-pasangan-untuk-hubungan-makin-hangat</t>
         </is>
       </c>
     </row>
@@ -1854,11 +1847,11 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>1. Daftar Tempat Wisata Semarang untuk Keluarga dan Anak (AI Citation Score: 10/10 | Type: Recommendation)
-2. Wisata Edukasi dan Alam di Semarang yang Ramah Anak (AI Citation Score: 9/10 | Type: Recommendation)
-3. Wisata Semarang Gratis dan Murah untuk Liburan Keluarga (AI Citation Score: 9/10 | Type: Recommendation)
-4. Perbandingan Harga Tiket, Jam Buka, dan Fasilitas Ramah Anak (AI Citation Score: 9/10 | Type: Comparative)
-5. Tips Liburan Keluarga ke Semarang: Rute, Waktu Terbaik, dan Itinerary 1–2 Hari (AI Citation Score: 8/10 | Type: Procedural)</t>
+          <t>1. Daftar Tempat Wisata Semarang untuk Keluarga dan Anak
+2. Wisata Edukasi dan Alam di Semarang yang Ramah Anak
+3. Wisata Semarang Gratis dan Murah untuk Liburan Keluarga
+4. Perbandingan Harga Tiket, Jam Buka, dan Fasilitas Ramah Anak
+5. Tips Liburan Keluarga ke Semarang: Rute, Waktu Terbaik, dan Itinerary 1–2 Hari</t>
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr">
@@ -1875,10 +1868,9 @@
       </c>
       <c r="G32" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: manfaat hidup rukun dalam keluarga → URL: https://motherandbeyond.id/read/25369/6-manfaat-hidup-rukun-dalam-keluarga-bisa-mengurangi-stres
-2. Anchor: kata-kata motivasi untuk keluarga → URL: https://motherandbeyond.id/read/27023/70-kata-kata-motivasi-untuk-keluarga-yang-menginspirasi
-3. Anchor: ide menu bekal anak → URL: https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi
-Limited relevant internal link available from Ahrefs export.</t>
+          <t>1. https://motherandbeyond.id/read/25369/6-manfaat-hidup-rukun-dalam-keluarga-bisa-mengurangi-stres
+2. https://motherandbeyond.id/read/27023/70-kata-kata-motivasi-untuk-keluarga-yang-menginspirasi
+3. https://motherandbeyond.id/read/26863/ide-menu-bekal-sekolah-anak-sd-selama-seminggu-yang-praktis-enak-dan-bergizi</t>
         </is>
       </c>
     </row>
@@ -1898,11 +1890,11 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>1. Apa Itu Kesundulan dan Bagaimana Mitosnya pada Bayi? (AI Citation Score: 9/10 | Type: Definitional)
-2. Ciri-Ciri Bayi yang Ibunya Hamil Lagi Menurut Kepercayaan Masyarakat (AI Citation Score: 8/10 | Type: Factual)
-3. Penjelasan Medis: Perubahan Rasa dan Produksi ASI saat Ibu Hamil Lagi (AI Citation Score: 10/10 | Type: Factual)
-4. Tanda-Tanda Ibu Menyusui Hamil Lagi yang Perlu Diwaspadai (AI Citation Score: 10/10 | Type: Factual)
-5. Bolehkah Tetap Menyusui saat Hamil? Panduan Aman untuk Ibu dan Bayi (AI Citation Score: 9/10 | Type: Procedural)</t>
+          <t>1. Apa Itu Kesundulan dan Bagaimana Mitosnya pada Bayi?
+2. Ciri-Ciri Bayi yang Ibunya Hamil Lagi Menurut Kepercayaan Masyarakat
+3. Penjelasan Medis: Perubahan Rasa dan Produksi ASI saat Ibu Hamil Lagi
+4. Tanda-Tanda Ibu Menyusui Hamil Lagi yang Perlu Diwaspadai
+5. Bolehkah Tetap Menyusui saat Hamil? Panduan Aman untuk Ibu dan Bayi</t>
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr">
@@ -1919,11 +1911,11 @@
       </c>
       <c r="G33" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: tips ketika ibu kesundulan → URL: https://motherandbeyond.id/read/7558/3-tips-ketika-ibu-kesundulan
-2. Anchor: tanda-tanda hamil setelah lepas KB suntik → URL: https://motherandbeyond.id/read/27846/tanda-tanda-hamil-setelah-lepas-kb-suntik-1-bulan-cek-ciri-cirinya
-3. Anchor: apakah ibu menyusui boleh minum es → URL: https://motherandbeyond.id/read/28033/apakah-ibu-menyusui-boleh-minum-es-ini-jawabannya
-4. Anchor: pantangan ibu baru melahirkan sebelum 40 hari → URL: https://motherandbeyond.id/read/26873/pantangan-ibu-baru-melahirkan-sebelum-40-hari-mitos-atau-fakta-medis
-5. Anchor: balita cengeng dan cara mengatasinya → URL: https://motherandbeyond.id/read/17263/balita-cengeng-ini-penyebab-dan-cara-mengatasinya</t>
+          <t>1. https://motherandbeyond.id/read/7558/3-tips-ketika-ibu-kesundulan
+2. https://motherandbeyond.id/read/27846/tanda-tanda-hamil-setelah-lepas-kb-suntik-1-bulan-cek-ciri-cirinya
+3. https://motherandbeyond.id/read/28033/apakah-ibu-menyusui-boleh-minum-es-ini-jawabannya
+4. https://motherandbeyond.id/read/26873/pantangan-ibu-baru-melahirkan-sebelum-40-hari-mitos-atau-fakta-medis
+5. https://motherandbeyond.id/read/17263/balita-cengeng-ini-penyebab-dan-cara-mengatasinya</t>
         </is>
       </c>
     </row>
@@ -1943,11 +1935,11 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>1. Dampak Anak yang Sering Dimarahi pada Kesehatan Mentalnya (AI Citation Score: 9/10 | Type: Factual)
-2. Tanda Anak Mengalami Luka Emosional Akibat Sering Dimarahi (AI Citation Score: 10/10 | Type: Factual)
-3. Cara Memperbaiki Mental Anak yang Sering Dimarahi: Langkah demi Langkah (AI Citation Score: 10/10 | Type: Procedural)
-4. Contoh Kalimat Meminta Maaf dan Membangun Kembali Kepercayaan Anak (AI Citation Score: 8/10 | Type: Recommendation)
-5. Kapan Anak Perlu Dibawa ke Psikolog? (AI Citation Score: 9/10 | Type: Procedural)</t>
+          <t>1. Dampak Anak yang Sering Dimarahi pada Kesehatan Mentalnya
+2. Tanda Anak Mengalami Luka Emosional Akibat Sering Dimarahi
+3. Cara Memperbaiki Mental Anak yang Sering Dimarahi: Langkah demi Langkah
+4. Contoh Kalimat Meminta Maaf dan Membangun Kembali Kepercayaan Anak
+5. Kapan Anak Perlu Dibawa ke Psikolog?</t>
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr">
@@ -1964,11 +1956,11 @@
       </c>
       <c r="G34" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: mimpi memarahi anak sendiri → URL: https://motherandbeyond.id/read/27661/mimpi-memarahi-anak-sendiri-ini-artinya-moms
-2. Anchor: cara mengatasi balita yang suka melawan → URL: https://motherandbeyond.id/read/20609/cara-tepat-mengatasi-balita-yang-suka-melawan-orang-tua
-3. Anchor: balita suka memukul diri sendiri → URL: https://motherandbeyond.id/read/17397/balita-suka-memukul-diri-sendiri-ini-penyebabnya-moms
-4. Anchor: balita cengeng dan cara mengatasinya → URL: https://motherandbeyond.id/read/17263/balita-cengeng-ini-penyebab-dan-cara-mengatasinya
-5. Anchor: manfaat hidup rukun dalam keluarga → URL: https://motherandbeyond.id/read/25369/6-manfaat-hidup-rukun-dalam-keluarga-bisa-mengurangi-stres</t>
+          <t>1. https://motherandbeyond.id/read/27661/mimpi-memarahi-anak-sendiri-ini-artinya-moms
+2. https://motherandbeyond.id/read/20609/cara-tepat-mengatasi-balita-yang-suka-melawan-orang-tua
+3. https://motherandbeyond.id/read/17397/balita-suka-memukul-diri-sendiri-ini-penyebabnya-moms
+4. https://motherandbeyond.id/read/17263/balita-cengeng-ini-penyebab-dan-cara-mengatasinya
+5. https://motherandbeyond.id/read/25369/6-manfaat-hidup-rukun-dalam-keluarga-bisa-mengurangi-stres</t>
         </is>
       </c>
     </row>
@@ -1988,11 +1980,11 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>1. Kenapa Orang Tua Mudah Emosi Saat Mendampingi Anak Belajar? (AI Citation Score: 8/10 | Type: Factual)
-2. Siapkan Diri Dulu: Teknik Menenangkan Emosi Sebelum Sesi Belajar (AI Citation Score: 9/10 | Type: Procedural)
-3. Cara Mengajari Anak Belajar Tanpa Emosi: Strategi Sesi Singkat dan Pilihan (AI Citation Score: 10/10 | Type: Procedural)
-4. Kalimat yang Sebaiknya Diucapkan vs Dihindari Saat Anak Kesulitan (AI Citation Score: 9/10 | Type: Comparative)
-5. Menyesuaikan Cara Belajar dengan Gaya Belajar dan Usia Anak (AI Citation Score: 8/10 | Type: Recommendation)</t>
+          <t>1. Kenapa Orang Tua Mudah Emosi Saat Mendampingi Anak Belajar?
+2. Siapkan Diri Dulu: Teknik Menenangkan Emosi Sebelum Sesi Belajar
+3. Cara Mengajari Anak Belajar Tanpa Emosi: Strategi Sesi Singkat dan Pilihan
+4. Kalimat yang Sebaiknya Diucapkan vs Dihindari Saat Anak Kesulitan
+5. Menyesuaikan Cara Belajar dengan Gaya Belajar dan Usia Anak</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
@@ -2009,10 +2001,10 @@
       </c>
       <c r="G35" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: kata-kata motivasi untuk anak SD → URL: https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
-2. Anchor: 100 soal pengetahuan umum SD → URL: https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
-3. Anchor: mimpi memarahi anak sendiri → URL: https://motherandbeyond.id/read/27661/mimpi-memarahi-anak-sendiri-ini-artinya-moms
-4. Anchor: ciri anak hiperaktif → URL: https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun</t>
+          <t>1. https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
+2. https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
+3. https://motherandbeyond.id/read/27661/mimpi-memarahi-anak-sendiri-ini-artinya-moms
+4. https://motherandbeyond.id/read/27646/balita-terlihat-sangat-aktif-kenali-ciri-anak-hiperaktif-usia-2-tahun</t>
         </is>
       </c>
     </row>
@@ -2032,11 +2024,11 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>1. Makna Kata-Kata Ayah bagi Tumbuh Kembang Anak (AI Citation Score: 7/10 | Type: Factual)
-2. Kata Mutiara Ayah kepada Anak yang Menyentuh Hati (AI Citation Score: 10/10 | Type: Recommendation)
-3. Kata Bijak Ayah untuk Anak Laki-Laki tentang Kehidupan dan Tanggung Jawab (AI Citation Score: 9/10 | Type: Recommendation)
-4. Kata-Kata Ayah untuk Anak Perempuan Penuh Nasihat dan Kasih Sayang (AI Citation Score: 9/10 | Type: Recommendation)
-5. Kata Mutiara Ayah Islami dan Versi Bahasa Inggris Beserta Artinya (AI Citation Score: 8/10 | Type: Recommendation)</t>
+          <t>1. Makna Kata-Kata Ayah bagi Tumbuh Kembang Anak
+2. Kata Mutiara Ayah kepada Anak yang Menyentuh Hati
+3. Kata Bijak Ayah untuk Anak Laki-Laki tentang Kehidupan dan Tanggung Jawab
+4. Kata-Kata Ayah untuk Anak Perempuan Penuh Nasihat dan Kasih Sayang
+5. Kata Mutiara Ayah Islami dan Versi Bahasa Inggris Beserta Artinya</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
@@ -2053,12 +2045,12 @@
       </c>
       <c r="G36" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: kata-kata doa untuk anak perempuan tersayang → URL: https://motherandbeyond.id/read/27727/50-kata-kata-doa-untuk-anak-perempuan-tersayang-agar-tumbuh-bahagia
-2. Anchor: ucapan ulang tahun untuk anak laki-laki → URL: https://motherandbeyond.id/read/27213/50-ucapan-ulang-tahun-untuk-anak-laki-laki-yang-menyentuh-hati
-3. Anchor: kata mutiara islami untuk anak perempuan → URL: https://motherandbeyond.id/read/17989/15-kata-mutiara-untuk-anak-perempuan-islami
-4. Anchor: kata-kata ibu rindu anak → URL: https://motherandbeyond.id/read/27467/50-kata-kata-ibu-rindu-anak-yang-menyentuh-dan-penuh-makna
-5. Anchor: kata-kata motivasi untuk keluarga → URL: https://motherandbeyond.id/read/27023/70-kata-kata-motivasi-untuk-keluarga-yang-menginspirasi
-6. Anchor: mimpi ayah meninggal → URL: https://motherandbeyond.id/read/28191/mimpi-ayah-meninggal-dan-anda-menangis-pertanda-apa</t>
+          <t>1. https://motherandbeyond.id/read/27727/50-kata-kata-doa-untuk-anak-perempuan-tersayang-agar-tumbuh-bahagia
+2. https://motherandbeyond.id/read/27213/50-ucapan-ulang-tahun-untuk-anak-laki-laki-yang-menyentuh-hati
+3. https://motherandbeyond.id/read/17989/15-kata-mutiara-untuk-anak-perempuan-islami
+4. https://motherandbeyond.id/read/27467/50-kata-kata-ibu-rindu-anak-yang-menyentuh-dan-penuh-makna
+5. https://motherandbeyond.id/read/27023/70-kata-kata-motivasi-untuk-keluarga-yang-menginspirasi
+6. https://motherandbeyond.id/read/28191/mimpi-ayah-meninggal-dan-anda-menangis-pertanda-apa</t>
         </is>
       </c>
     </row>
@@ -2078,11 +2070,11 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>1. Manfaat Lomba Kreatif untuk Tumbuh Kembang Anak (AI Citation Score: 7/10 | Type: Factual)
-2. Ide Lomba Anak-Anak yang Unik dan Kreatif untuk Mengasah Imajinasi (AI Citation Score: 10/10 | Type: Recommendation)
-3. Lomba Fisik yang Seru, Lucu, dan Aman untuk Anak (AI Citation Score: 9/10 | Type: Recommendation)
-4. Ide Lomba Sesuai Usia: Balita, TK, dan SD (AI Citation Score: 9/10 | Type: Comparative)
-5. Cara Menyiapkan Lomba Anak: Alat, Aturan, dan Penilaian (AI Citation Score: 8/10 | Type: Procedural)</t>
+          <t>1. Manfaat Lomba Kreatif untuk Tumbuh Kembang Anak
+2. Ide Lomba Anak-Anak yang Unik dan Kreatif untuk Mengasah Imajinasi
+3. Lomba Fisik yang Seru, Lucu, dan Aman untuk Anak
+4. Ide Lomba Sesuai Usia: Balita, TK, dan SD
+5. Cara Menyiapkan Lomba Anak: Alat, Aturan, dan Penilaian</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -2099,10 +2091,10 @@
       </c>
       <c r="G37" s="3" t="inlineStr">
         <is>
-          <t>1. Anchor: soal pengetahuan umum SD dan jawabannya → URL: https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
-2. Anchor: kata-kata motivasi untuk anak SD → URL: https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
-3. Anchor: manfaat pop it fidget toy → URL: https://motherandbeyond.id/read/23087/bukan-mainan-biasa-ini-manfaat-dari-pop-it-fidget-toy-buat-anak
-4. Anchor: ucapan ulang tahun untuk anak laki-laki → URL: https://motherandbeyond.id/read/27213/50-ucapan-ulang-tahun-untuk-anak-laki-laki-yang-menyentuh-hati</t>
+          <t>1. https://motherandbeyond.id/read/28616/100-soal-pengetahuan-umum-sd-dan-jawabannya-bikin-anak-makin-cerdas
+2. https://motherandbeyond.id/read/27464/50-kata-kata-motivasi-untuk-anak-sd-agar-semangat-belajar
+3. https://motherandbeyond.id/read/23087/bukan-mainan-biasa-ini-manfaat-dari-pop-it-fidget-toy-buat-anak
+4. https://motherandbeyond.id/read/27213/50-ucapan-ulang-tahun-untuk-anak-laki-laki-yang-menyentuh-hati</t>
         </is>
       </c>
     </row>

</xml_diff>